<commit_message>
Ready-to-edit inputs rebuilt: half-hour starts and 11H/3OFF limit rows appear
The seven workbooks users fill in were never rebuilt after the template
gained these rows. Rebuilt with tools/build_input_template.py (135 parsed
fields verified identical per workbook) and checked independently: same
contract fingerprint, demand, shrinkage, roster, preferences and shift
library. Protected RC9.1 baselines untouched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MH973LepRRvS7jQvRfGiqr
</commit_message>
<xml_diff>
--- a/packages/rc9_2_2_production/inputs/ready_to_edit/AE_AR_B2B_WEEKLY_INPUT.xlsx
+++ b/packages/rc9_2_2_production/inputs/ready_to_edit/AE_AR_B2B_WEEKLY_INPUT.xlsx
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="E10" s="24">
-        <f>IF(Instructions!C35&lt;&gt;"Yes","Not used (Fixed Request Use = No)",IF(SUMPRODUCT(('Fixed Request'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Fixed Request'!$B$3:$B$302)=0))=0,"OK  every name is on the roster","! "&amp;SUMPRODUCT(('Fixed Request'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Fixed Request'!$B$3:$B$302)=0))&amp;" name(s) not on the roster"))</f>
+        <f>IF(Instructions!C37&lt;&gt;"Yes","Not used (Fixed Request Use = No)",IF(SUMPRODUCT(('Fixed Request'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Fixed Request'!$B$3:$B$302)=0))=0,"OK  every name is on the roster","! "&amp;SUMPRODUCT(('Fixed Request'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Fixed Request'!$B$3:$B$302)=0))&amp;" name(s) not on the roster"))</f>
         <v/>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="E11" s="24">
-        <f>IF(SUMPRODUCT(('Previous week scheduled'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Previous week scheduled'!$B$3:$B$302)=0)*ISERROR(SEARCH('Previous week scheduled'!$B$3:$B$302,"|"&amp;Instructions!C39&amp;"|")))=0,"OK  every name is on the roster or listed as departed","! "&amp;SUMPRODUCT(('Previous week scheduled'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Previous week scheduled'!$B$3:$B$302)=0)*ISERROR(SEARCH('Previous week scheduled'!$B$3:$B$302,"|"&amp;Instructions!C39&amp;"|")))&amp;" name(s) not on the roster: list them in Known Departed Associates if they left")</f>
+        <f>IF(SUMPRODUCT(('Previous week scheduled'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Previous week scheduled'!$B$3:$B$302)=0)*ISERROR(SEARCH('Previous week scheduled'!$B$3:$B$302,"|"&amp;Instructions!C41&amp;"|")))=0,"OK  every name is on the roster or listed as departed","! "&amp;SUMPRODUCT(('Previous week scheduled'!$B$3:$B$302&lt;&gt;"")*(COUNTIF('Schedule'!$D$3:$D$302,'Previous week scheduled'!$B$3:$B$302)=0)*ISERROR(SEARCH('Previous week scheduled'!$B$3:$B$302,"|"&amp;Instructions!C41&amp;"|")))&amp;" name(s) not on the roster: list them in Known Departed Associates if they left")</f>
         <v/>
       </c>
     </row>
@@ -2105,8 +2105,23 @@
     <cfRule type="expression" priority="2" dxfId="6">
       <formula>UPPER(TRIM(D3))="LEAVE"</formula>
     </cfRule>
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>UPPER(TRIM(D3))="OFF"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="6">
+      <formula>UPPER(TRIM(D3))="LEAVE"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="6">
+    <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="This name is not on this week's roster. If the person has left, also list them in Instructions &gt; Known Departed Associates." prompt="Pick a name from this week's roster." type="list" errorStyle="warning">
+      <formula1>'Schedule'!$D$3:$D$302</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3:C302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="This language is not on the Language Setup tab. Keep it only if that is intended." type="list" errorStyle="warning">
+      <formula1>'Language Setup'!$A$3:$A$42</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="Not in this week's Shift Library. Keep it only if it really was last Saturday's shift (HH:MM - HH:MM)." prompt="OFF, Leave or a shift from the Shift Library." type="list" errorStyle="warning">
+      <formula1>'Validation Lists'!$C$3:$C$69</formula1>
+    </dataValidation>
     <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="This name is not on this week's roster. If the person has left, also list them in Instructions &gt; Known Departed Associates." prompt="Pick a name from this week's roster." type="list" errorStyle="warning">
       <formula1>'Schedule'!$D$3:$D$302</formula1>
     </dataValidation>
@@ -2430,8 +2445,29 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="6">
+  <dataValidations count="12">
     <dataValidation sqref="J3 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid coverage days" error="Choose a listed day or range, or type a supported value such as Sun-Thu." type="list" errorStyle="stop">
+      <formula1>"All,Weekdays,Weekends,Sun-Thu,Mon-Fri,Sun,Mon,Tue,Wed,Thu,Fri,Sat"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B3:B42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. A time such as 08:00. The window may cross midnight." prompt="A time such as 08:00. The window may cross midnight." type="time" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.999988426</formula2>
+    </dataValidation>
+    <dataValidation sqref="C3:C42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. A time such as 08:00. The window may cross midnight." prompt="A time such as 08:00. The window may cross midnight." type="time" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.999988426</formula2>
+    </dataValidation>
+    <dataValidation sqref="E3:E42" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. People of this language needed at all times in the window (whole number)." prompt="People of this language needed at all times in the window (whole number)." type="whole" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>500</formula2>
+    </dataValidation>
+    <dataValidation sqref="I3:I42" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid coverage days" error="Choose a listed day or range, or type a supported value such as Sun-Thu." type="list" errorStyle="stop">
       <formula1>"All,Weekdays,Weekends,Sun-Thu,Mon-Fri,Sun,Mon,Tue,Wed,Thu,Fri,Sat"</formula1>
     </dataValidation>
     <dataValidation sqref="B3:B42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. A time such as 08:00. The window may cross midnight." prompt="A time such as 08:00. The window may cross midnight." type="time" errorStyle="stop" operator="between">
@@ -5688,7 +5724,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H98" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H98" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>100000</formula2>
@@ -7111,7 +7151,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H98" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.9999</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H98" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>0.9999</formula2>
@@ -8143,7 +8187,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -8504,132 +8548,124 @@
     <row r="29" ht="20" customHeight="1" s="18">
       <c r="B29" s="42" t="inlineStr">
         <is>
-          <t>Strict OFF Count</t>
-        </is>
-      </c>
-      <c r="C29" s="43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Max 11H/3OFF Associates</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="inlineStr"/>
       <c r="D29" s="44" t="inlineStr">
         <is>
-          <t>Yes = exactly two OFF days (three with 11H/3OFF) per person.</t>
+          <t>Blank = engine default. Used only when Use 11H/3OFF is Yes: the most associates who may work the 11-hour, three-OFF-day pattern this week (e.g. 2). Blank = no limit.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" s="18">
       <c r="B30" s="42" t="inlineStr">
         <is>
-          <t>Separate OFF Days</t>
+          <t>Strict OFF Count</t>
         </is>
       </c>
       <c r="C30" s="43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D30" s="44" t="inlineStr">
         <is>
-          <t>Yes = a person's OFF days may be apart. No = they must be together.</t>
+          <t>Yes = exactly two OFF days (three with 11H/3OFF) per person.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" s="18">
       <c r="B31" s="42" t="inlineStr">
         <is>
-          <t>Rest Gap Hours</t>
-        </is>
-      </c>
-      <c r="C31" s="47" t="n">
-        <v>12</v>
+          <t>Separate OFF Days</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="D31" s="44" t="inlineStr">
         <is>
-          <t>Minimum hours between the end of one shift and the start of the next.</t>
+          <t>Yes = a person's OFF days may be apart. No = they must be together.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" s="18">
       <c r="B32" s="42" t="inlineStr">
         <is>
+          <t>Rest Gap Hours</t>
+        </is>
+      </c>
+      <c r="C32" s="47" t="n">
+        <v>12</v>
+      </c>
+      <c r="D32" s="44" t="inlineStr">
+        <is>
+          <t>Minimum hours between the end of one shift and the start of the next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" s="18">
+      <c r="B33" s="42" t="inlineStr">
+        <is>
           <t>Count of Different Shifts Per week</t>
         </is>
       </c>
-      <c r="C32" s="45" t="n">
+      <c r="C33" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D32" s="44" t="inlineStr">
+      <c r="D33" s="44" t="inlineStr">
         <is>
           <t>Most different shifts one person may get in a week (1 to 7).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="40" t="inlineStr">
+    <row r="34" ht="20" customHeight="1" s="18">
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>Allow Half-Hour Starts</t>
+        </is>
+      </c>
+      <c r="C34" s="43" t="inlineStr"/>
+      <c r="D34" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Yes = each shift may also start 30 minutes later, used only where full-hour starts cannot cover demand; marked in the output. Blank or No = full-hour starts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="40" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="B34" s="41" t="n"/>
-      <c r="C34" s="41" t="n"/>
-      <c r="D34" s="41" t="n"/>
-    </row>
-    <row r="35" ht="20" customHeight="1" s="18">
-      <c r="B35" s="42" t="inlineStr">
-        <is>
-          <t>Fixed Request Use</t>
-        </is>
-      </c>
-      <c r="C35" s="43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D35" s="44" t="inlineStr">
-        <is>
-          <t>Yes = apply the Fixed Request tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1" s="18">
-      <c r="B36" s="42" t="inlineStr">
-        <is>
-          <t>Hard OFF Preferences</t>
-        </is>
-      </c>
-      <c r="C36" s="43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D36" s="44" t="inlineStr">
-        <is>
-          <t>Yes = OFF requests on the Preference tab are always granted.</t>
-        </is>
-      </c>
+      <c r="B36" s="41" t="n"/>
+      <c r="C36" s="41" t="n"/>
+      <c r="D36" s="41" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1" s="18">
       <c r="B37" s="42" t="inlineStr">
         <is>
-          <t>Leave Enabled</t>
+          <t>Fixed Request Use</t>
         </is>
       </c>
       <c r="C37" s="43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D37" s="44" t="inlineStr">
         <is>
-          <t>Yes = Leave on the Preference tab is honoured.</t>
+          <t>Yes = apply the Fixed Request tab.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1" s="18">
       <c r="B38" s="42" t="inlineStr">
         <is>
-          <t>Use Preferences</t>
+          <t>Hard OFF Preferences</t>
         </is>
       </c>
       <c r="C38" s="43" t="inlineStr">
@@ -8639,338 +8675,372 @@
       </c>
       <c r="D38" s="44" t="inlineStr">
         <is>
-          <t>Yes = try to give people their preferred shifts.</t>
+          <t>Yes = OFF requests on the Preference tab are always granted.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" s="18">
       <c r="B39" s="42" t="inlineStr">
         <is>
+          <t>Leave Enabled</t>
+        </is>
+      </c>
+      <c r="C39" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>Yes = Leave on the Preference tab is honoured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" s="18">
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>Use Preferences</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>Yes = try to give people their preferred shifts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="18">
+      <c r="B41" s="42" t="inlineStr">
+        <is>
           <t>Known Departed Associates</t>
         </is>
       </c>
-      <c r="C39" s="43" t="inlineStr"/>
-      <c r="D39" s="44" t="inlineStr">
+      <c r="C41" s="43" t="inlineStr"/>
+      <c r="D41" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. Names on last week's tab who have left, separated by ; (Start Here lists any missing).</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="40" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="40" t="inlineStr">
         <is>
           <t>Opening Guard   (click + on the left to open)</t>
         </is>
       </c>
-      <c r="B41" s="41" t="n"/>
-      <c r="C41" s="41" t="n"/>
-      <c r="D41" s="41" t="n"/>
-    </row>
-    <row r="42" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B42" s="42" t="inlineStr">
-        <is>
-          <t>Opening Guard Enabled</t>
-        </is>
-      </c>
-      <c r="C42" s="43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D42" s="44" t="inlineStr">
-        <is>
-          <t>Yes = keep enough people on at the start of each day.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B43" s="42" t="inlineStr">
-        <is>
-          <t>Opening Minimum FTE</t>
-        </is>
-      </c>
-      <c r="C43" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="44" t="inlineStr">
-        <is>
-          <t>People needed at opening (whole number).</t>
-        </is>
-      </c>
+      <c r="B43" s="41" t="n"/>
+      <c r="C43" s="41" t="n"/>
+      <c r="D43" s="41" t="n"/>
     </row>
     <row r="44" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B44" s="42" t="inlineStr">
         <is>
+          <t>Opening Guard Enabled</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D44" s="44" t="inlineStr">
+        <is>
+          <t>Yes = keep enough people on at the start of each day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B45" s="42" t="inlineStr">
+        <is>
+          <t>Opening Minimum FTE</t>
+        </is>
+      </c>
+      <c r="C45" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="44" t="inlineStr">
+        <is>
+          <t>People needed at opening (whole number).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B46" s="42" t="inlineStr">
+        <is>
           <t>Opening Guard Intervals</t>
         </is>
       </c>
-      <c r="C44" s="45" t="n">
+      <c r="C46" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D44" s="44" t="inlineStr">
+      <c r="D46" s="44" t="inlineStr">
         <is>
           <t>How many opening intervals the guard covers.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="40" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="40" t="inlineStr">
         <is>
           <t>Breaks</t>
         </is>
       </c>
-      <c r="B46" s="41" t="n"/>
-      <c r="C46" s="41" t="n"/>
-      <c r="D46" s="41" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" s="18">
-      <c r="B47" s="42" t="inlineStr">
-        <is>
-          <t>Short Break Count</t>
-        </is>
-      </c>
-      <c r="C47" s="43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" s="44" t="inlineStr">
-        <is>
-          <t>Short breaks per shift.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1" s="18">
-      <c r="B48" s="42" t="inlineStr">
-        <is>
-          <t>Short Break Duration Minutes</t>
-        </is>
-      </c>
-      <c r="C48" s="43" t="n">
-        <v>15</v>
-      </c>
-      <c r="D48" s="44" t="inlineStr">
-        <is>
-          <t>Length of each short break.</t>
-        </is>
-      </c>
+      <c r="B48" s="41" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="41" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1" s="18">
       <c r="B49" s="42" t="inlineStr">
         <is>
-          <t>Lunch Count</t>
+          <t>Short Break Count</t>
         </is>
       </c>
       <c r="C49" s="43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" s="44" t="inlineStr">
         <is>
-          <t>Lunches per shift.</t>
+          <t>Short breaks per shift.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1" s="18">
       <c r="B50" s="42" t="inlineStr">
         <is>
-          <t>Lunch Duration Minutes</t>
+          <t>Short Break Duration Minutes</t>
         </is>
       </c>
       <c r="C50" s="43" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D50" s="44" t="inlineStr">
         <is>
-          <t>Length of each lunch.</t>
+          <t>Length of each short break.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1" s="18">
       <c r="B51" s="42" t="inlineStr">
         <is>
-          <t>Break Preferred Gap Minutes</t>
-        </is>
-      </c>
-      <c r="C51" s="45" t="n">
-        <v>150</v>
+          <t>Lunch Count</t>
+        </is>
+      </c>
+      <c r="C51" s="43" t="n">
+        <v>1</v>
       </c>
       <c r="D51" s="44" t="inlineStr">
         <is>
-          <t>Ideal minutes between two breaks.</t>
+          <t>Lunches per shift.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1" s="18">
       <c r="B52" s="42" t="inlineStr">
         <is>
-          <t>Break Absolute Minimum Gap Minutes</t>
-        </is>
-      </c>
-      <c r="C52" s="45" t="n">
-        <v>60</v>
+          <t>Lunch Duration Minutes</t>
+        </is>
+      </c>
+      <c r="C52" s="43" t="n">
+        <v>30</v>
       </c>
       <c r="D52" s="44" t="inlineStr">
         <is>
-          <t>Two breaks are never closer than this.</t>
+          <t>Length of each lunch.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1" s="18">
       <c r="B53" s="42" t="inlineStr">
         <is>
-          <t>Break Normal Maximum Gap Minutes</t>
+          <t>Break Preferred Gap Minutes</t>
         </is>
       </c>
       <c r="C53" s="45" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="D53" s="44" t="inlineStr">
         <is>
-          <t>Two breaks are normally no further apart than this.</t>
+          <t>Ideal minutes between two breaks.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1" s="18">
       <c r="B54" s="42" t="inlineStr">
         <is>
+          <t>Break Absolute Minimum Gap Minutes</t>
+        </is>
+      </c>
+      <c r="C54" s="45" t="n">
+        <v>60</v>
+      </c>
+      <c r="D54" s="44" t="inlineStr">
+        <is>
+          <t>Two breaks are never closer than this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1" s="18">
+      <c r="B55" s="42" t="inlineStr">
+        <is>
+          <t>Break Normal Maximum Gap Minutes</t>
+        </is>
+      </c>
+      <c r="C55" s="45" t="n">
+        <v>210</v>
+      </c>
+      <c r="D55" s="44" t="inlineStr">
+        <is>
+          <t>Two breaks are normally no further apart than this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1" s="18">
+      <c r="B56" s="42" t="inlineStr">
+        <is>
           <t>Allow Back-to-Back Breaks</t>
         </is>
       </c>
-      <c r="C54" s="43" t="inlineStr">
+      <c r="C56" s="43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D54" s="44" t="inlineStr">
+      <c r="D56" s="44" t="inlineStr">
         <is>
           <t>Yes = a break may directly follow another.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="40" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="40" t="inlineStr">
         <is>
           <t>Language / Skill</t>
         </is>
       </c>
-      <c r="B56" s="41" t="n"/>
-      <c r="C56" s="41" t="n"/>
-      <c r="D56" s="41" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1" s="18">
-      <c r="B57" s="42" t="inlineStr">
+      <c r="B58" s="41" t="n"/>
+      <c r="C58" s="41" t="n"/>
+      <c r="D58" s="41" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1" s="18">
+      <c r="B59" s="42" t="inlineStr">
         <is>
           <t>Language Working Window</t>
         </is>
       </c>
-      <c r="C57" s="43" t="inlineStr"/>
-      <c r="D57" s="44" t="inlineStr">
+      <c r="C59" s="43" t="inlineStr"/>
+      <c r="D59" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. OFF = language hours set minimums only. The other choices also limit when each language may work (guide 3.7).</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="40" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="40" t="inlineStr">
         <is>
           <t>Exception Policy</t>
         </is>
       </c>
-      <c r="B59" s="41" t="n"/>
-      <c r="C59" s="41" t="n"/>
-      <c r="D59" s="41" t="n"/>
-    </row>
-    <row r="60" ht="20" customHeight="1" s="18">
-      <c r="B60" s="42" t="inlineStr">
+      <c r="B61" s="41" t="n"/>
+      <c r="C61" s="41" t="n"/>
+      <c r="D61" s="41" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1" s="18">
+      <c r="B62" s="42" t="inlineStr">
         <is>
           <t>Critical Coverage No-Break Exception Enabled</t>
         </is>
       </c>
-      <c r="C60" s="43" t="inlineStr">
+      <c r="C62" s="43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D60" s="44" t="inlineStr">
+      <c r="D62" s="44" t="inlineStr">
         <is>
           <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="20" customHeight="1" s="18">
-      <c r="B61" s="42" t="inlineStr">
+    <row r="63" ht="20" customHeight="1" s="18">
+      <c r="B63" s="42" t="inlineStr">
         <is>
           <t>Critical Coverage No-Break Max Associate-Days</t>
         </is>
       </c>
-      <c r="C61" s="45" t="n">
+      <c r="C63" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D61" s="44" t="inlineStr">
+      <c r="D63" s="44" t="inlineStr">
         <is>
           <t>Most person-days that may skip a break. Above 0 when enabled.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="40" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="40" t="inlineStr">
         <is>
           <t>Release Quality   (click + on the left to open)</t>
         </is>
       </c>
-      <c r="B63" s="41" t="n"/>
-      <c r="C63" s="41" t="n"/>
-      <c r="D63" s="41" t="n"/>
-    </row>
-    <row r="64" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B64" s="42" t="inlineStr">
-        <is>
-          <t>Production Quality Gate Mode</t>
-        </is>
-      </c>
-      <c r="C64" s="43" t="inlineStr">
-        <is>
-          <t>Warn</t>
-        </is>
-      </c>
-      <c r="D64" s="44" t="inlineStr">
-        <is>
-          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B65" s="42" t="inlineStr">
-        <is>
-          <t>Minimum After Break Target Ratio</t>
-        </is>
-      </c>
-      <c r="C65" s="46" t="inlineStr"/>
-      <c r="D65" s="44" t="inlineStr">
-        <is>
-          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
-        </is>
-      </c>
+      <c r="B65" s="41" t="n"/>
+      <c r="C65" s="41" t="n"/>
+      <c r="D65" s="41" t="n"/>
     </row>
     <row r="66" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B66" s="42" t="inlineStr">
         <is>
-          <t>Protected Before80 Minimum Intervals</t>
-        </is>
-      </c>
-      <c r="C66" s="45" t="inlineStr"/>
+          <t>Production Quality Gate Mode</t>
+        </is>
+      </c>
+      <c r="C66" s="43" t="inlineStr">
+        <is>
+          <t>Warn</t>
+        </is>
+      </c>
       <c r="D66" s="44" t="inlineStr">
         <is>
-          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
         </is>
       </c>
     </row>
     <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B67" s="42" t="inlineStr">
         <is>
+          <t>Minimum After Break Target Ratio</t>
+        </is>
+      </c>
+      <c r="C67" s="46" t="inlineStr"/>
+      <c r="D67" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B68" s="42" t="inlineStr">
+        <is>
+          <t>Protected Before80 Minimum Intervals</t>
+        </is>
+      </c>
+      <c r="C68" s="45" t="inlineStr"/>
+      <c r="D68" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B69" s="42" t="inlineStr">
+        <is>
           <t>Protected After80 Minimum Intervals</t>
         </is>
       </c>
-      <c r="C67" s="45" t="inlineStr"/>
-      <c r="D67" s="44" t="inlineStr">
+      <c r="C69" s="45" t="inlineStr"/>
+      <c r="D69" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. Optional. Intervals that must reach 80% after breaks.</t>
         </is>
@@ -8981,7 +9051,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="30">
+  <dataValidations count="31">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 80 characters." prompt="Up to 80 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>80</formula1>
     </dataValidation>
@@ -8989,7 +9059,7 @@
       <formula1>1</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C8 C16 C20 C22 C28 C29 C30 C35 C36 C37 C38 C42 C54 C60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
@@ -9024,65 +9094,69 @@
     <dataValidation sqref="C27" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Shift lengths allowed. 10.5 h or more needs Use 11H/3OFF = Yes." type="list" errorStyle="stop">
       <formula1>'Validation Lists'!$A$3:$A$33</formula1>
     </dataValidation>
-    <dataValidation sqref="C31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0 to 24." prompt="Enter a number from 0 to 24." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 5000." prompt="Enter a whole number from 1 to 5000." type="whole" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>5000</formula2>
+    </dataValidation>
+    <dataValidation sqref="C32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0 to 24." prompt="Enter a number from 0 to 24." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
-    <dataValidation sqref="C32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 7." prompt="Enter a whole number from 1 to 7." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 7." prompt="Enter a whole number from 1 to 7." type="whole" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>7</formula2>
     </dataValidation>
-    <dataValidation sqref="C39" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 2000 characters." prompt="Up to 2000 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
+    <dataValidation sqref="C41" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 2000 characters." prompt="Up to 2000 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>2000</formula1>
     </dataValidation>
-    <dataValidation sqref="C43" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 500." prompt="Enter a whole number from 0 to 500." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C45" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 500." prompt="Enter a whole number from 0 to 500." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>500</formula2>
     </dataValidation>
-    <dataValidation sqref="C44" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 96." prompt="Enter a whole number from 0 to 96." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C46" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 96." prompt="Enter a whole number from 0 to 96." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>96</formula2>
     </dataValidation>
-    <dataValidation sqref="C47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"0,1,2,3,4"</formula1>
     </dataValidation>
-    <dataValidation sqref="C48 C50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C50 C52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"15,30,45,60"</formula1>
     </dataValidation>
-    <dataValidation sqref="C49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"0,1,2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 720." prompt="Enter a whole number from 0 to 720." type="whole" errorStyle="stop" operator="between">
-      <formula1>0</formula1>
-      <formula2>720</formula2>
-    </dataValidation>
-    <dataValidation sqref="C52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 720." prompt="Enter a whole number from 0 to 720." type="whole" errorStyle="stop" operator="between">
-      <formula1>0</formula1>
-      <formula2>720</formula2>
     </dataValidation>
     <dataValidation sqref="C53" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 720." prompt="Enter a whole number from 0 to 720." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>720</formula2>
     </dataValidation>
-    <dataValidation sqref="C57" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C54" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 720." prompt="Enter a whole number from 0 to 720." type="whole" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>720</formula2>
+    </dataValidation>
+    <dataValidation sqref="C55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 720." prompt="Enter a whole number from 0 to 720." type="whole" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>720</formula2>
+    </dataValidation>
+    <dataValidation sqref="C59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"OFF,MINIMUM_ROWS,ALL_ROWS,REQUIRED_LANGUAGE_ONLY"</formula1>
     </dataValidation>
-    <dataValidation sqref="C61" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Warn,Fail,Off"</formula1>
     </dataValidation>
-    <dataValidation sqref="C65" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C68" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
-    <dataValidation sqref="C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
@@ -11712,7 +11786,19 @@
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="8">
+    <dataValidation sqref="D3:D302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This name is already on the roster. One row per person." prompt="One row per person. Names must match the other tabs." type="custom" errorStyle="stop">
+      <formula1>COUNTIF($D$3:$D$302,D3)&lt;=1</formula1>
+    </dataValidation>
+    <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This employee ID is already on the roster." prompt="Employee ID, once per person." type="custom" errorStyle="stop">
+      <formula1>COUNTIF($B$3:$B$302,B3)&lt;=1</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3:F302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="This language is not on the Language Setup tab. Keep it only if that is intended." prompt="Pick the language from Language Setup." type="list" errorStyle="warning">
+      <formula1>'Language Setup'!$A$3:$A$42</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G302 H3:H302 I3:I302 J3:J302 K3:K302 L3:L302 M3:M302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="OFF, Leave or a shift from the Shift Library." type="list" errorStyle="stop">
+      <formula1>'Validation Lists'!$B$3:$B$68</formula1>
+    </dataValidation>
     <dataValidation sqref="D3:D302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This name is already on the roster. One row per person." prompt="One row per person. Names must match the other tabs." type="custom" errorStyle="stop">
       <formula1>COUNTIF($D$3:$D$302,D3)&lt;=1</formula1>
     </dataValidation>
@@ -12471,7 +12557,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>100000</formula2>
@@ -13222,7 +13312,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H50" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H50" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Required FTE for this interval. 0 or more; blank = no demand." prompt="Required FTE for this interval. 0 or more; blank = no demand." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>100000</formula2>
@@ -13972,7 +14066,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.9999</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>0.9999</formula2>
@@ -14723,7 +14821,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:H50" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.9999</formula2>
+    </dataValidation>
     <dataValidation sqref="B3:H50" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Shrinkage as a ratio (0.08) or percent (8%). Below 100%." prompt="Shrinkage as a ratio (0.08) or percent (8%). Below 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>0.9999</formula2>
@@ -15368,8 +15470,23 @@
     <cfRule type="expression" priority="2" dxfId="6">
       <formula>UPPER(TRIM(C3))="LEAVE"</formula>
     </cfRule>
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>UPPER(TRIM(C3))="OFF"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="6">
+      <formula>UPPER(TRIM(C3))="LEAVE"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="6">
+    <dataValidation sqref="A3:A302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Pick a name from this week's roster." type="list" errorStyle="stop">
+      <formula1>'Schedule'!$D$3:$D$302</formula1>
+    </dataValidation>
+    <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Please check this value" error="This language is not on the Language Setup tab. Keep it only if that is intended." type="list" errorStyle="warning">
+      <formula1>'Language Setup'!$A$3:$A$42</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3:C302 D3:D302 E3:E302 F3:F302 G3:G302 H3:H302 I3:I302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="OFF, Leave or a shift from the Shift Library." type="list" errorStyle="stop">
+      <formula1>'Validation Lists'!$B$3:$B$68</formula1>
+    </dataValidation>
     <dataValidation sqref="A3:A302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Pick a name from this week's roster." type="list" errorStyle="stop">
       <formula1>'Schedule'!$D$3:$D$302</formula1>
     </dataValidation>
@@ -15558,8 +15675,26 @@
     <cfRule type="expression" priority="2" dxfId="6">
       <formula>UPPER(TRIM(D3))="LEAVE"</formula>
     </cfRule>
+    <cfRule type="expression" priority="3" dxfId="5">
+      <formula>UPPER(TRIM(D3))="OFF"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="6">
+      <formula>UPPER(TRIM(D3))="LEAVE"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="8">
+    <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Pick a name from this week's roster." type="list" errorStyle="stop">
+      <formula1>'Schedule'!$D$3:$D$302</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D302 E3:E302 F3:F302 G3:G302 H3:H302 I3:I302 J3:J302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="OFF, Leave or a shift from the Shift Library." type="list" errorStyle="stop">
+      <formula1>'Validation Lists'!$B$3:$B$68</formula1>
+    </dataValidation>
+    <dataValidation sqref="A3:A302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Yes = apply this row. No = ignore it." type="list" errorStyle="stop">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3:C302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Optional. People with the same group number work the same shifts." prompt="Optional. People with the same group number work the same shifts." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
+      <formula1>50</formula1>
+    </dataValidation>
     <dataValidation sqref="B3:B302" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." prompt="Pick a name from this week's roster." type="list" errorStyle="stop">
       <formula1>'Schedule'!$D$3:$D$302</formula1>
     </dataValidation>

</xml_diff>